<commit_message>
Add calculation rules to specifications
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
+++ b/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2204" uniqueCount="721">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -2177,6 +2177,45 @@
   </si>
   <si>
     <t>Identity: [extendedCurrencyCreditInstitutionTurnoverBasedAssetsForCalculationOfGreenAssetRatioTurnoverBasedTotalGrossCarryingAmount]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentEligible]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichUseOfProceeds]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichTransitional]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichEnabling]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyAssetManagementAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalAssetManagementBreakdownOfTheNumeratorOfTheKpiTurnoverBasedShareOfTurnoverBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyAssetManagementAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalAssetManagementBreakdownOfTheNumeratorOfTheKpiCapexBasedShareOfCapexBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyEligibleActivities,extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyAlignedActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiums,extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyEligibleActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyEligibleActivities,extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyAlignedActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ComplementToPercent: [extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyEligibleActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyInsuranceReinsuranceAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalInsuranceReinsuranceBreakdownOfTheNumeratorOfTheKpiTurnoverBasedShareOfTurnoverBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyInsuranceReinsuranceAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalInsuranceReinsuranceBreakdownOfTheNumeratorOfTheKpiCapexBasedShareOfCapexBasedKpiInPercentAligned]</t>
   </si>
 </sst>
 </file>
@@ -4054,6 +4093,9 @@
         <v>57</v>
       </c>
       <c r="P10" s="16"/>
+      <c r="Q10" s="16" t="s">
+        <v>708</v>
+      </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" s="53">
@@ -4094,6 +4136,9 @@
         <v>57</v>
       </c>
       <c r="P11" s="16"/>
+      <c r="Q11" s="16" t="s">
+        <v>709</v>
+      </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
@@ -4134,6 +4179,9 @@
         <v>57</v>
       </c>
       <c r="P12" s="24"/>
+      <c r="Q12" s="16" t="s">
+        <v>710</v>
+      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" s="25" t="s">
@@ -4174,6 +4222,9 @@
         <v>57</v>
       </c>
       <c r="P13" s="16"/>
+      <c r="Q13" s="16" t="s">
+        <v>711</v>
+      </c>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="82" t="s">
@@ -4214,6 +4265,9 @@
         <v>57</v>
       </c>
       <c r="P14" s="23"/>
+      <c r="Q14" s="16" t="s">
+        <v>712</v>
+      </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="25">
@@ -6686,6 +6740,9 @@
       </c>
       <c r="O79" s="16"/>
       <c r="P79" s="16"/>
+      <c r="Q79" s="16" t="s">
+        <v>713</v>
+      </c>
     </row>
     <row r="80" spans="1:17" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="84">
@@ -6724,6 +6781,9 @@
       </c>
       <c r="O80" s="63"/>
       <c r="P80" s="63"/>
+      <c r="Q80" s="16" t="s">
+        <v>714</v>
+      </c>
     </row>
     <row r="81" spans="1:17" ht="14.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A81" s="38">
@@ -7794,6 +7854,9 @@
       </c>
       <c r="O108" s="44"/>
       <c r="P108" s="44"/>
+      <c r="Q108" s="16" t="s">
+        <v>715</v>
+      </c>
     </row>
     <row r="109" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="43">
@@ -7832,6 +7895,9 @@
       </c>
       <c r="O109" s="44"/>
       <c r="P109" s="44"/>
+      <c r="Q109" s="16" t="s">
+        <v>716</v>
+      </c>
     </row>
     <row r="110" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="43">
@@ -7904,6 +7970,9 @@
       </c>
       <c r="O111" s="44"/>
       <c r="P111" s="44"/>
+      <c r="Q111" s="16" t="s">
+        <v>717</v>
+      </c>
     </row>
     <row r="112" spans="1:16" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="34">
@@ -7940,6 +8009,9 @@
       </c>
       <c r="O112" s="59"/>
       <c r="P112" s="59"/>
+      <c r="Q112" s="16" t="s">
+        <v>718</v>
+      </c>
     </row>
     <row r="113" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A113" s="43">
@@ -8056,6 +8128,9 @@
       </c>
       <c r="O115" s="16"/>
       <c r="P115" s="16"/>
+      <c r="Q115" s="16" t="s">
+        <v>719</v>
+      </c>
     </row>
     <row r="116" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="34">
@@ -8094,6 +8169,9 @@
       </c>
       <c r="O116" s="63"/>
       <c r="P116" s="63"/>
+      <c r="Q116" s="16" t="s">
+        <v>720</v>
+      </c>
     </row>
     <row r="117" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A117" s="43">

</xml_diff>

<commit_message>
Dala 7482 support for calculated fields mapping into old frameworks (#2051)
Co-authored-by: SiegfriedSobkowiak <71646830+SiegfriedSobkowiak@users.noreply.github.com>
Co-authored-by: StephanWezorke <186339469+StephanWezorke@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
+++ b/dataland-framework-toolbox/inputs/eu-taxonomy-financials/eu-taxonomy-financials.xlsx
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2204" uniqueCount="721">
   <si>
     <t>Field Identifier</t>
   </si>
@@ -2177,6 +2177,45 @@
   </si>
   <si>
     <t>Identity: [extendedCurrencyCreditInstitutionTurnoverBasedAssetsForCalculationOfGreenAssetRatioTurnoverBasedTotalGrossCarryingAmount]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentEligible]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichUseOfProceeds]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichTransitional]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyCreditInstitutionAssetsForCalculationOfGreenAssetRatioTotalGrossCarryingAmount,extendedDecimalCreditInstitutionTurnoverBasedGreenAssetRatioStockSubstantialContributionToAnyOfTheSixEnvironmentalObjectivesInPercentOfWhichEnabling]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyAssetManagementAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalAssetManagementBreakdownOfTheNumeratorOfTheKpiTurnoverBasedShareOfTurnoverBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyAssetManagementAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalAssetManagementBreakdownOfTheNumeratorOfTheKpiCapexBasedShareOfCapexBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyEligibleActivities,extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyAlignedActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiums,extendedCurrencyInsuranceReinsuranceTotalOfAbsolutePremiumsOfTaxonomyEligibleActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtraction: [extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyEligibleActivities,extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyAlignedActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ComplementToPercent: [extendedDecimalInsuranceReinsuranceProportionOfAbsolutePremiumsOfTaxonomyEligibleActivities]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyInsuranceReinsuranceAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalInsuranceReinsuranceBreakdownOfTheNumeratorOfTheKpiTurnoverBasedShareOfTurnoverBasedKpiInPercentAligned]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MultiplicationByPercent: [extendedCurrencyInsuranceReinsuranceAssetUnderManagementAssetsCoveredByTheKpiMonetaryAmount,extendedDecimalInsuranceReinsuranceBreakdownOfTheNumeratorOfTheKpiCapexBasedShareOfCapexBasedKpiInPercentAligned]</t>
   </si>
 </sst>
 </file>
@@ -4054,6 +4093,9 @@
         <v>57</v>
       </c>
       <c r="P10" s="16"/>
+      <c r="Q10" s="16" t="s">
+        <v>708</v>
+      </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A11" s="53">
@@ -4094,6 +4136,9 @@
         <v>57</v>
       </c>
       <c r="P11" s="16"/>
+      <c r="Q11" s="16" t="s">
+        <v>709</v>
+      </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
@@ -4134,6 +4179,9 @@
         <v>57</v>
       </c>
       <c r="P12" s="24"/>
+      <c r="Q12" s="16" t="s">
+        <v>710</v>
+      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A13" s="25" t="s">
@@ -4174,6 +4222,9 @@
         <v>57</v>
       </c>
       <c r="P13" s="16"/>
+      <c r="Q13" s="16" t="s">
+        <v>711</v>
+      </c>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="82" t="s">
@@ -4214,6 +4265,9 @@
         <v>57</v>
       </c>
       <c r="P14" s="23"/>
+      <c r="Q14" s="16" t="s">
+        <v>712</v>
+      </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A15" s="25">
@@ -6686,6 +6740,9 @@
       </c>
       <c r="O79" s="16"/>
       <c r="P79" s="16"/>
+      <c r="Q79" s="16" t="s">
+        <v>713</v>
+      </c>
     </row>
     <row r="80" spans="1:17" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="84">
@@ -6724,6 +6781,9 @@
       </c>
       <c r="O80" s="63"/>
       <c r="P80" s="63"/>
+      <c r="Q80" s="16" t="s">
+        <v>714</v>
+      </c>
     </row>
     <row r="81" spans="1:17" ht="14.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A81" s="38">
@@ -7794,6 +7854,9 @@
       </c>
       <c r="O108" s="44"/>
       <c r="P108" s="44"/>
+      <c r="Q108" s="16" t="s">
+        <v>715</v>
+      </c>
     </row>
     <row r="109" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="43">
@@ -7832,6 +7895,9 @@
       </c>
       <c r="O109" s="44"/>
       <c r="P109" s="44"/>
+      <c r="Q109" s="16" t="s">
+        <v>716</v>
+      </c>
     </row>
     <row r="110" spans="1:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="43">
@@ -7904,6 +7970,9 @@
       </c>
       <c r="O111" s="44"/>
       <c r="P111" s="44"/>
+      <c r="Q111" s="16" t="s">
+        <v>717</v>
+      </c>
     </row>
     <row r="112" spans="1:16" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="34">
@@ -7940,6 +8009,9 @@
       </c>
       <c r="O112" s="59"/>
       <c r="P112" s="59"/>
+      <c r="Q112" s="16" t="s">
+        <v>718</v>
+      </c>
     </row>
     <row r="113" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A113" s="43">
@@ -8056,6 +8128,9 @@
       </c>
       <c r="O115" s="16"/>
       <c r="P115" s="16"/>
+      <c r="Q115" s="16" t="s">
+        <v>719</v>
+      </c>
     </row>
     <row r="116" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="34">
@@ -8094,6 +8169,9 @@
       </c>
       <c r="O116" s="63"/>
       <c r="P116" s="63"/>
+      <c r="Q116" s="16" t="s">
+        <v>720</v>
+      </c>
     </row>
     <row r="117" spans="1:17" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A117" s="43">

</xml_diff>